<commit_message>
preparing new version - step 1
</commit_message>
<xml_diff>
--- a/external/linelist_passwords.xlsx
+++ b/external/linelist_passwords.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/komlaviamevoin/Documents/Projects/outbreak-tools/misc/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/komlaviamevoin/Unsync-Working-Folders/outbreak-tools/external/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DDE3ADB-1E27-7A48-8401-C5D6D164F050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{131CFB49-3465-7040-BF72-E365107199DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="500" windowWidth="50120" windowHeight="28300" xr2:uid="{9E4A9F11-575A-4617-A17F-5F801F975382}"/>
+    <workbookView xWindow="1080" yWindow="620" windowWidth="50120" windowHeight="27220" xr2:uid="{9E4A9F11-575A-4617-A17F-5F801F975382}"/>
   </bookViews>
   <sheets>
     <sheet name="version_a" sheetId="2" r:id="rId1"/>
@@ -26,25 +26,25 @@
     <definedName name="DESIGNS_LIST">[1]LinelistStyle!$C$1:$E$1</definedName>
     <definedName name="hf_concat">[1]!T_HF[hf_concat]</definedName>
     <definedName name="LangDictList">[1]!T_LanguageDictionary[LangDict]</definedName>
-    <definedName name="RNG_DebuggingPassword">version_a!$I$1</definedName>
-    <definedName name="RNG_DebugMode">version_a!$K$1</definedName>
+    <definedName name="RNG_DebuggingPassword">version_a!$B$5</definedName>
+    <definedName name="RNG_DebugMode">version_a!$B$6</definedName>
     <definedName name="RNG_DesignLL">[1]Main!$F$8</definedName>
     <definedName name="RNG_DictionaryLanguage">[1]!T_SelectedLLLanguages[linelist dictionary language]</definedName>
     <definedName name="RNG_GeoLangCode">[1]Geo!$BI$1</definedName>
-    <definedName name="RNG_LabPrivateKey">version_a!$A$3</definedName>
-    <definedName name="RNG_LabPublicKey">version_a!$A$2</definedName>
+    <definedName name="RNG_LabPrivateKey">version_a!$A$4</definedName>
+    <definedName name="RNG_LabPublicKey">version_a!$A$3</definedName>
     <definedName name="RNG_LLLanguage">[1]LinelistTranslation!$E$285</definedName>
     <definedName name="RNG_LLLanguageCode">[1]LinelistTranslation!$F$285</definedName>
     <definedName name="RNG_MainLangCode">[1]DesignerTranslation!$C$133</definedName>
-    <definedName name="RNG_PrivateKey">version_a!$B$3</definedName>
-    <definedName name="RNG_PublicKey">version_a!$B$2</definedName>
+    <definedName name="RNG_PrivateKey">version_a!$B$4</definedName>
+    <definedName name="RNG_PublicKey">version_a!$B$3</definedName>
     <definedName name="RNG_TargetVersion">#REF!</definedName>
-    <definedName name="RNG_Version">version_a!$M$1</definedName>
+    <definedName name="RNG_Version">version_a!$B$7</definedName>
     <definedName name="T_NAMES_GEO">[1]!T_NAMES[[#All],[ENG]:[ARA]]</definedName>
     <definedName name="TABLES_STYLES_LIST">[1]LinelistStyle!$K$2:$K$63</definedName>
     <definedName name="UserLangList">[1]!T_Lang[Languages]</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0" calcOnSave="0"/>
+  <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>PublicKeys</t>
   </si>
@@ -84,12 +84,30 @@
   <si>
     <t>d0099</t>
   </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>DrawObjects</t>
+  </si>
+  <si>
+    <t>DeleteRows</t>
+  </si>
+  <si>
+    <t>Debugging Password</t>
+  </si>
+  <si>
+    <t>Debug Mode</t>
+  </si>
+  <si>
+    <t>Password version</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -100,13 +118,37 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -119,8 +161,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -129,30 +183,157 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
+      <left/>
+      <right style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <top/>
+      <bottom style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
+      <left style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
+      <right style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </right>
+      <top style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </right>
+      <top style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right/>
+      <top style="hair">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </right>
+      <top style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right/>
+      <top style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </right>
+      <top style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right/>
+      <top style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </left>
+      <right style="thick">
+        <color theme="4" tint="-0.499984740745262"/>
+      </right>
+      <top style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
+      </top>
+      <bottom style="dotted">
+        <color theme="4" tint="0.39994506668294322"/>
       </bottom>
       <diagonal/>
     </border>
@@ -160,67 +341,331 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="15">
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
       <fill>
-        <patternFill patternType="none">
+        <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right/>
+        <top style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <border>
+        <bottom style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
-        <patternFill patternType="none">
+        <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </vertical>
+        <horizontal style="hair">
+          <color theme="4" tint="0.39994506668294322"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right/>
+        <top style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
+      <border>
+        <bottom style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -234,17 +679,33 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color theme="0"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
       <fill>
-        <patternFill patternType="none">
+        <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor theme="4" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </left>
+        <right style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </vertical>
+        <horizontal style="dotted">
+          <color theme="4" tint="0.39994506668294322"/>
+        </horizontal>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -645,20 +1106,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{15C73615-5A09-40E1-B98F-78CEAF10D6ED}" name="T_Keys" displayName="T_Keys" ref="D1:E3" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3" tableBorderDxfId="2">
-  <autoFilter ref="D1:E3" xr:uid="{219C3623-9437-428F-A255-77C479205693}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{15C73615-5A09-40E1-B98F-78CEAF10D6ED}" name="T_Keys" displayName="T_Keys" ref="D3:E5" totalsRowShown="0" headerRowDxfId="14" dataDxfId="12" headerRowBorderDxfId="13" tableBorderDxfId="11" totalsRowBorderDxfId="10">
+  <autoFilter ref="D3:E5" xr:uid="{219C3623-9437-428F-A255-77C479205693}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{F4F0D697-EBF0-4AD3-9E0B-DA0C051C99AA}" name="PublicKeys" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{8487113E-D4E0-4C5D-AC03-6F221B9C307D}" name="PrivateKeys" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{F4F0D697-EBF0-4AD3-9E0B-DA0C051C99AA}" name="PublicKeys" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{8487113E-D4E0-4C5D-AC03-6F221B9C307D}" name="PrivateKeys" dataDxfId="8"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{FDF55B82-B6F9-5E4E-B9DC-B965B34FF5B0}" name="T_ProtectedSheets" displayName="T_ProtectedSheets" ref="H3:J4" totalsRowShown="0" headerRowDxfId="7" dataDxfId="5" headerRowBorderDxfId="6" tableBorderDxfId="4" totalsRowBorderDxfId="3">
+  <autoFilter ref="H3:J4" xr:uid="{FDF55B82-B6F9-5E4E-B9DC-B965B34FF5B0}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{2D940D81-E5F7-6B41-955E-D0507E179E5A}" name="ID" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{5F9015B6-359A-5640-82CD-481A266C39A8}" name="DrawObjects" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{C7801953-0082-6346-83AE-ED081EB985FF}" name="DeleteRows" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -696,7 +1169,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -802,7 +1275,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -944,7 +1417,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -953,74 +1426,101 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC8B9CDE-01BA-491C-9C6E-778CF09A3690}">
   <sheetPr codeName="Sheet12"/>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A3:O8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="1" max="1" width="26.1640625" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="4" max="4" width="23.33203125" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
+    <col min="8" max="10" width="35.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="D1" s="2" t="s">
+    <row r="3" spans="1:15" ht="21" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="17">
+        <v>1234</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="I1">
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="M3" s="8"/>
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="17">
         <v>1234</v>
       </c>
-      <c r="K1" t="s">
+      <c r="D4" s="10">
+        <v>1234</v>
+      </c>
+      <c r="E4" s="11">
+        <v>1234</v>
+      </c>
+      <c r="H4" s="14"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="16"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="17">
+        <v>1234</v>
+      </c>
+      <c r="D5" s="12">
+        <v>6789</v>
+      </c>
+      <c r="E5" s="13">
+        <v>6789</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="7" t="s">
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3">
-        <v>1234</v>
-      </c>
-      <c r="D2">
-        <v>1234</v>
-      </c>
-      <c r="E2">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="4">
-        <v>1234</v>
-      </c>
-      <c r="D3">
-        <v>6789</v>
-      </c>
-      <c r="E3">
-        <v>6789</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="5"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B6" s="6"/>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B8" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>